<commit_message>
Auto-derive input hints from constraints; add header-cell Note API
Input hints: every constrained column now surfaces its rule proactively as an
Excel input-message tooltip (shown on cell select), derived from the same
metadata as the validation error — "Select one of: ...", "Enter a number
between X and Y.", "This field is required.". An explicit InputMessage still
wins, and the bare ISNUMBER type check is deliberately not surfaced (noise on
every numeric cell). Opt out per column with DisableInputMessage.
Notes: new Note(prop, text) attaches a legacy red-triangle comment to a
column's heading cell. Unlike an input hint it stays visible on hover under
sheet protection, so it is the place to explain why a column is locked. Emits
the comments part + VML + <legacyDrawing>; validates clean against the
Office2019 schema. Works on data-bound, dictionary, and template sheets.
Both features are additive (no WordTableBuilder/ctor changes), so existing
Parchment builds keep working.
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/ColumnAttributeTests.Test.verified.xlsx
+++ b/src/Excelsior.Tests/ColumnAttributeTests.Test.verified.xlsx
@@ -154,13 +154,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="custom" allowBlank="0" showErrorMessage="1" errorTitle="Invalid value" error="Must be a number." sqref="A2:A3">
+    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a number." prompt="This field is required." sqref="A2:A3">
       <formula1>ISNUMBER(A2)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="0" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." sqref="B2:B3">
+    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="This field is required." sqref="B2:B3">
       <formula1>LEN(TRIM(B2))&gt;0</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="0" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." sqref="D2:D3">
+    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="This field is required." sqref="D2:D3">
       <formula1>LEN(TRIM(D2))&gt;0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>